<commit_message>
chore: run 2026-03-01 14:46 — histórico, dashboard e Excel atualizados
</commit_message>
<xml_diff>
--- a/logs/Consolidado_01_03_2026.xlsx
+++ b/logs/Consolidado_01_03_2026.xlsx
@@ -602,10 +602,10 @@
         <v>151</v>
       </c>
       <c r="C2" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="D2" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="E2" t="n">
         <v>4</v>
@@ -621,10 +621,10 @@
         <v>66</v>
       </c>
       <c r="C3" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="D3" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="E3" t="n">
         <v>1</v>
@@ -640,10 +640,10 @@
         <v>85</v>
       </c>
       <c r="C4" t="n">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="D4" t="n">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="E4" t="n">
         <v>3</v>
@@ -659,10 +659,10 @@
         <v>72</v>
       </c>
       <c r="C5" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="D5" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="E5" t="n">
         <v>3</v>
@@ -1392,40 +1392,40 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="7" t="inlineStr">
-        <is>
-          <t>01/03/2026</t>
-        </is>
-      </c>
-      <c r="B18" s="7" t="inlineStr">
+      <c r="A18" s="3" t="inlineStr">
+        <is>
+          <t>01/03/2026</t>
+        </is>
+      </c>
+      <c r="B18" s="3" t="inlineStr">
         <is>
           <t>Avène</t>
         </is>
       </c>
-      <c r="C18" s="7" t="inlineStr">
+      <c r="C18" s="3" t="inlineStr">
         <is>
           <t>Cicalfate+ Purifying Cleansing Gel
 Gel de Limpeza Purificante da Pele Irritada
 200 ml</t>
         </is>
       </c>
-      <c r="D18" s="7" t="inlineStr">
+      <c r="D18" s="3" t="inlineStr">
         <is>
           <t>https://wells.pt/cicalfate-purifying-cleansing-gel-7632460.html</t>
         </is>
       </c>
-      <c r="E18" s="7" t="inlineStr"/>
-      <c r="F18" s="8" t="inlineStr">
-        <is>
-          <t>Out of Stock</t>
-        </is>
-      </c>
-      <c r="G18" s="7" t="inlineStr">
+      <c r="E18" s="3" t="inlineStr"/>
+      <c r="F18" s="4" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
+      <c r="G18" s="3" t="inlineStr">
         <is>
           <t>7632460</t>
         </is>
       </c>
-      <c r="H18" s="7" t="inlineStr">
+      <c r="H18" s="3" t="inlineStr">
         <is>
           <t>25%</t>
         </is>
@@ -2330,40 +2330,40 @@
       </c>
     </row>
     <row r="41">
-      <c r="A41" s="7" t="inlineStr">
-        <is>
-          <t>01/03/2026</t>
-        </is>
-      </c>
-      <c r="B41" s="7" t="inlineStr">
+      <c r="A41" s="5" t="inlineStr">
+        <is>
+          <t>01/03/2026</t>
+        </is>
+      </c>
+      <c r="B41" s="5" t="inlineStr">
         <is>
           <t>Avène</t>
         </is>
       </c>
-      <c r="C41" s="7" t="inlineStr">
+      <c r="C41" s="5" t="inlineStr">
         <is>
           <t>Cold Cream Nousishing Lip Balm
 Bálsamo Reparador de Lábios Secos
 4gr</t>
         </is>
       </c>
-      <c r="D41" s="7" t="inlineStr">
+      <c r="D41" s="5" t="inlineStr">
         <is>
           <t>https://wells.pt/cold-cream-nousishing-lip-balm-3000767.html</t>
         </is>
       </c>
-      <c r="E41" s="7" t="inlineStr"/>
-      <c r="F41" s="8" t="inlineStr">
-        <is>
-          <t>Out of Stock</t>
-        </is>
-      </c>
-      <c r="G41" s="7" t="inlineStr">
+      <c r="E41" s="5" t="inlineStr"/>
+      <c r="F41" s="6" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
+      <c r="G41" s="5" t="inlineStr">
         <is>
           <t>3000767</t>
         </is>
       </c>
-      <c r="H41" s="7" t="inlineStr">
+      <c r="H41" s="5" t="inlineStr">
         <is>
           <t>25%</t>
         </is>
@@ -5964,7 +5964,7 @@
       </c>
       <c r="G131" s="3" t="inlineStr">
         <is>
-          <t>3000998</t>
+          <t>3000993</t>
         </is>
       </c>
       <c r="H131" s="3" t="inlineStr">
@@ -7495,40 +7495,40 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="7" t="inlineStr">
-        <is>
-          <t>01/03/2026</t>
-        </is>
-      </c>
-      <c r="B10" s="7" t="inlineStr">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>01/03/2026</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="inlineStr">
         <is>
           <t>Ducray</t>
         </is>
       </c>
-      <c r="C10" s="7" t="inlineStr">
+      <c r="C10" s="5" t="inlineStr">
         <is>
           <t>Creme Palpebral Eczema Dexyane Med
 Creme Eczema da Pálpebra
 15 ml</t>
         </is>
       </c>
-      <c r="D10" s="7" t="inlineStr">
+      <c r="D10" s="5" t="inlineStr">
         <is>
           <t>https://wells.pt/creme-palpebral-eczema-dexyane-med-7024952.html</t>
         </is>
       </c>
-      <c r="E10" s="7" t="inlineStr"/>
-      <c r="F10" s="8" t="inlineStr">
-        <is>
-          <t>Out of Stock</t>
-        </is>
-      </c>
-      <c r="G10" s="7" t="inlineStr">
+      <c r="E10" s="5" t="inlineStr"/>
+      <c r="F10" s="6" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
+      <c r="G10" s="5" t="inlineStr">
         <is>
           <t>7024952</t>
         </is>
       </c>
-      <c r="H10" s="7" t="inlineStr">
+      <c r="H10" s="5" t="inlineStr">
         <is>
           <t>25%</t>
         </is>
@@ -8921,40 +8921,40 @@
       </c>
     </row>
     <row r="45">
-      <c r="A45" s="7" t="inlineStr">
-        <is>
-          <t>01/03/2026</t>
-        </is>
-      </c>
-      <c r="B45" s="7" t="inlineStr">
+      <c r="A45" s="3" t="inlineStr">
+        <is>
+          <t>01/03/2026</t>
+        </is>
+      </c>
+      <c r="B45" s="3" t="inlineStr">
         <is>
           <t>Ducray</t>
         </is>
       </c>
-      <c r="C45" s="7" t="inlineStr">
+      <c r="C45" s="3" t="inlineStr">
         <is>
           <t>Keracnyl Mat 12H Oily Skin
 Gel Matificante Pele Oleosa Ação Anti-brilho
 30 ml</t>
         </is>
       </c>
-      <c r="D45" s="7" t="inlineStr">
+      <c r="D45" s="3" t="inlineStr">
         <is>
           <t>https://wells.pt/keracnyl-mat-12h-oily-skin-6037944.html</t>
         </is>
       </c>
-      <c r="E45" s="7" t="inlineStr"/>
-      <c r="F45" s="8" t="inlineStr">
-        <is>
-          <t>Out of Stock</t>
-        </is>
-      </c>
-      <c r="G45" s="7" t="inlineStr">
+      <c r="E45" s="3" t="inlineStr"/>
+      <c r="F45" s="4" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
+      <c r="G45" s="3" t="inlineStr">
         <is>
           <t>6037944</t>
         </is>
       </c>
-      <c r="H45" s="7" t="inlineStr">
+      <c r="H45" s="3" t="inlineStr">
         <is>
           <t>25%</t>
         </is>
@@ -9001,40 +9001,40 @@
       </c>
     </row>
     <row r="47">
-      <c r="A47" s="7" t="inlineStr">
-        <is>
-          <t>01/03/2026</t>
-        </is>
-      </c>
-      <c r="B47" s="7" t="inlineStr">
+      <c r="A47" s="3" t="inlineStr">
+        <is>
+          <t>01/03/2026</t>
+        </is>
+      </c>
+      <c r="B47" s="3" t="inlineStr">
         <is>
           <t>Ducray</t>
         </is>
       </c>
-      <c r="C47" s="7" t="inlineStr">
+      <c r="C47" s="3" t="inlineStr">
         <is>
           <t>Keracnyl Repair Baume Lèvres
 Bálsamo Lábios Gretados e Danificados Acne
 15 ml</t>
         </is>
       </c>
-      <c r="D47" s="7" t="inlineStr">
+      <c r="D47" s="3" t="inlineStr">
         <is>
           <t>https://wells.pt/keracnyl-repair-baume-levres-5410512.html</t>
         </is>
       </c>
-      <c r="E47" s="7" t="inlineStr"/>
-      <c r="F47" s="8" t="inlineStr">
-        <is>
-          <t>Out of Stock</t>
-        </is>
-      </c>
-      <c r="G47" s="7" t="inlineStr">
+      <c r="E47" s="3" t="inlineStr"/>
+      <c r="F47" s="4" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
+      <c r="G47" s="3" t="inlineStr">
         <is>
           <t>5410512</t>
         </is>
       </c>
-      <c r="H47" s="7" t="inlineStr">
+      <c r="H47" s="3" t="inlineStr">
         <is>
           <t>25%</t>
         </is>
@@ -9841,40 +9841,40 @@
       </c>
     </row>
     <row r="68">
-      <c r="A68" s="7" t="inlineStr">
-        <is>
-          <t>01/03/2026</t>
-        </is>
-      </c>
-      <c r="B68" s="7" t="inlineStr">
+      <c r="A68" s="5" t="inlineStr">
+        <is>
+          <t>01/03/2026</t>
+        </is>
+      </c>
+      <c r="B68" s="5" t="inlineStr">
         <is>
           <t>Ducray</t>
         </is>
       </c>
-      <c r="C68" s="7" t="inlineStr">
+      <c r="C68" s="5" t="inlineStr">
         <is>
           <t>Sensinol Shampooing Physioprotecteur
 Champô Calmante Couro Cabeludo Sensível
 400 ml</t>
         </is>
       </c>
-      <c r="D68" s="7" t="inlineStr">
+      <c r="D68" s="5" t="inlineStr">
         <is>
           <t>https://wells.pt/sensinol-shampooing-physioprotecteur-7646502.html</t>
         </is>
       </c>
-      <c r="E68" s="7" t="inlineStr"/>
-      <c r="F68" s="8" t="inlineStr">
-        <is>
-          <t>Out of Stock</t>
-        </is>
-      </c>
-      <c r="G68" s="7" t="inlineStr">
+      <c r="E68" s="5" t="inlineStr"/>
+      <c r="F68" s="6" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
+      <c r="G68" s="5" t="inlineStr">
         <is>
           <t>7646502</t>
         </is>
       </c>
-      <c r="H68" s="7" t="inlineStr">
+      <c r="H68" s="5" t="inlineStr">
         <is>
           <t>25%</t>
         </is>
@@ -10156,40 +10156,40 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="7" t="inlineStr">
-        <is>
-          <t>01/03/2026</t>
-        </is>
-      </c>
-      <c r="B2" s="7" t="inlineStr">
+      <c r="A2" s="3" t="inlineStr">
+        <is>
+          <t>01/03/2026</t>
+        </is>
+      </c>
+      <c r="B2" s="3" t="inlineStr">
         <is>
           <t>Klorane</t>
         </is>
       </c>
-      <c r="C2" s="7" t="inlineStr">
+      <c r="C2" s="3" t="inlineStr">
         <is>
           <t>Aquatic Mint Detox Dry Shampoo
 Champô Seco Menta BIO Detox Antipoluição
 150 ml</t>
         </is>
       </c>
-      <c r="D2" s="7" t="inlineStr">
+      <c r="D2" s="3" t="inlineStr">
         <is>
           <t>https://wells.pt/aquatic-mint-detox-dry-shampoo-7339166.html</t>
         </is>
       </c>
-      <c r="E2" s="7" t="inlineStr"/>
-      <c r="F2" s="8" t="inlineStr">
-        <is>
-          <t>Out of Stock</t>
-        </is>
-      </c>
-      <c r="G2" s="7" t="inlineStr">
+      <c r="E2" s="3" t="inlineStr"/>
+      <c r="F2" s="4" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
+      <c r="G2" s="3" t="inlineStr">
         <is>
           <t>7339166</t>
         </is>
       </c>
-      <c r="H2" s="7" t="inlineStr">
+      <c r="H2" s="3" t="inlineStr">
         <is>
           <t>25%</t>
         </is>
@@ -12963,86 +12963,86 @@
       </c>
     </row>
     <row r="71">
-      <c r="A71" s="7" t="inlineStr">
-        <is>
-          <t>01/03/2026</t>
-        </is>
-      </c>
-      <c r="B71" s="7" t="inlineStr">
+      <c r="A71" s="5" t="inlineStr">
+        <is>
+          <t>01/03/2026</t>
+        </is>
+      </c>
+      <c r="B71" s="5" t="inlineStr">
         <is>
           <t>Klorane</t>
         </is>
       </c>
-      <c r="C71" s="7" t="inlineStr">
+      <c r="C71" s="5" t="inlineStr">
         <is>
           <t>Nettle Oil Control Shampoo
 Champô Ortiga BIO Purifica Cabelo Oleoso</t>
         </is>
       </c>
-      <c r="D71" s="7" t="inlineStr">
+      <c r="D71" s="5" t="inlineStr">
         <is>
           <t>https://wells.pt/nettle-oil-control-shampoo-343980.html</t>
         </is>
       </c>
-      <c r="E71" s="7" t="inlineStr">
+      <c r="E71" s="5" t="inlineStr">
         <is>
           <t>400 ml</t>
         </is>
       </c>
-      <c r="F71" s="8" t="inlineStr">
-        <is>
-          <t>Out of Stock</t>
-        </is>
-      </c>
-      <c r="G71" s="7" t="inlineStr">
+      <c r="F71" s="6" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
+      <c r="G71" s="5" t="inlineStr">
         <is>
           <t>3688262</t>
         </is>
       </c>
-      <c r="H71" s="7" t="inlineStr">
+      <c r="H71" s="5" t="inlineStr">
         <is>
           <t>35%</t>
         </is>
       </c>
     </row>
     <row r="72">
-      <c r="A72" s="7" t="inlineStr">
-        <is>
-          <t>01/03/2026</t>
-        </is>
-      </c>
-      <c r="B72" s="7" t="inlineStr">
+      <c r="A72" s="3" t="inlineStr">
+        <is>
+          <t>01/03/2026</t>
+        </is>
+      </c>
+      <c r="B72" s="3" t="inlineStr">
         <is>
           <t>Klorane</t>
         </is>
       </c>
-      <c r="C72" s="7" t="inlineStr">
+      <c r="C72" s="3" t="inlineStr">
         <is>
           <t>Oat &amp; Ceramide Ultra-Gentle Dry Shampoo
 Champô Seco Aveia Spray Suave Cabelo Normal</t>
         </is>
       </c>
-      <c r="D72" s="7" t="inlineStr">
+      <c r="D72" s="3" t="inlineStr">
         <is>
           <t>https://wells.pt/oat-and-ceramide-ultra-gentle-dry-shampoo-341981.html</t>
         </is>
       </c>
-      <c r="E72" s="7" t="inlineStr">
+      <c r="E72" s="3" t="inlineStr">
         <is>
           <t>50 ml</t>
         </is>
       </c>
-      <c r="F72" s="8" t="inlineStr">
-        <is>
-          <t>Out of Stock</t>
-        </is>
-      </c>
-      <c r="G72" s="7" t="inlineStr">
+      <c r="F72" s="4" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
+      <c r="G72" s="3" t="inlineStr">
         <is>
           <t>7831152</t>
         </is>
       </c>
-      <c r="H72" s="7" t="inlineStr">
+      <c r="H72" s="3" t="inlineStr">
         <is>
           <t>25%</t>
         </is>
@@ -14039,40 +14039,40 @@
       </c>
     </row>
     <row r="97">
-      <c r="A97" s="7" t="inlineStr">
-        <is>
-          <t>01/03/2026</t>
-        </is>
-      </c>
-      <c r="B97" s="7" t="inlineStr">
+      <c r="A97" s="5" t="inlineStr">
+        <is>
+          <t>01/03/2026</t>
+        </is>
+      </c>
+      <c r="B97" s="5" t="inlineStr">
         <is>
           <t>Klorane</t>
         </is>
       </c>
-      <c r="C97" s="7" t="inlineStr">
+      <c r="C97" s="5" t="inlineStr">
         <is>
           <t>Tamanu &amp; Monoi Nutri-Repair Sun Conditioner
 Condicionador Protetor Solar para Cabelo
 200 ml</t>
         </is>
       </c>
-      <c r="D97" s="7" t="inlineStr">
+      <c r="D97" s="5" t="inlineStr">
         <is>
           <t>https://wells.pt/tamanu-and-monoi-nutri-repair-sun-conditioner-7396247.html</t>
         </is>
       </c>
-      <c r="E97" s="7" t="inlineStr"/>
-      <c r="F97" s="8" t="inlineStr">
-        <is>
-          <t>Out of Stock</t>
-        </is>
-      </c>
-      <c r="G97" s="7" t="inlineStr">
+      <c r="E97" s="5" t="inlineStr"/>
+      <c r="F97" s="6" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
+      <c r="G97" s="5" t="inlineStr">
         <is>
           <t>7396247</t>
         </is>
       </c>
-      <c r="H97" s="7" t="inlineStr">
+      <c r="H97" s="5" t="inlineStr">
         <is>
           <t>37%</t>
         </is>
@@ -14747,40 +14747,40 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="7" t="inlineStr">
-        <is>
-          <t>01/03/2026</t>
-        </is>
-      </c>
-      <c r="B12" s="7" t="inlineStr">
+      <c r="A12" s="3" t="inlineStr">
+        <is>
+          <t>01/03/2026</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="inlineStr">
         <is>
           <t>René Furterer</t>
         </is>
       </c>
-      <c r="C12" s="7" t="inlineStr">
+      <c r="C12" s="3" t="inlineStr">
         <is>
           <t>Astera Fresh Soothing Freshness Shampoo
 Champô Calmante Couro Cabeludo Irritado
 200 ml</t>
         </is>
       </c>
-      <c r="D12" s="7" t="inlineStr">
+      <c r="D12" s="3" t="inlineStr">
         <is>
           <t>https://wells.pt/astera-fresh-soothing-freshness-shampoo-5520033.html</t>
         </is>
       </c>
-      <c r="E12" s="7" t="inlineStr"/>
-      <c r="F12" s="8" t="inlineStr">
-        <is>
-          <t>Out of Stock</t>
-        </is>
-      </c>
-      <c r="G12" s="7" t="inlineStr">
+      <c r="E12" s="3" t="inlineStr"/>
+      <c r="F12" s="4" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
+      <c r="G12" s="3" t="inlineStr">
         <is>
           <t>5520033</t>
         </is>
       </c>
-      <c r="H12" s="7" t="inlineStr">
+      <c r="H12" s="3" t="inlineStr">
         <is>
           <t>25%</t>
         </is>
@@ -15152,40 +15152,40 @@
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="7" t="inlineStr">
-        <is>
-          <t>01/03/2026</t>
-        </is>
-      </c>
-      <c r="B22" s="7" t="inlineStr">
+      <c r="A22" s="5" t="inlineStr">
+        <is>
+          <t>01/03/2026</t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="inlineStr">
         <is>
           <t>René Furterer</t>
         </is>
       </c>
-      <c r="C22" s="7" t="inlineStr">
+      <c r="C22" s="5" t="inlineStr">
         <is>
           <t>Forticea Strengthening Revitalizing Shampoo
 Champô Fortificante Todos Tipos de Cabelo
 500 ml</t>
         </is>
       </c>
-      <c r="D22" s="7" t="inlineStr">
+      <c r="D22" s="5" t="inlineStr">
         <is>
           <t>https://wells.pt/forticea-strengthening-revitalizing-shampoo-8602496.html</t>
         </is>
       </c>
-      <c r="E22" s="7" t="inlineStr"/>
-      <c r="F22" s="8" t="inlineStr">
-        <is>
-          <t>Out of Stock</t>
-        </is>
-      </c>
-      <c r="G22" s="7" t="inlineStr">
+      <c r="E22" s="5" t="inlineStr"/>
+      <c r="F22" s="6" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
+      <c r="G22" s="5" t="inlineStr">
         <is>
           <t>8602496</t>
         </is>
       </c>
-      <c r="H22" s="7" t="inlineStr">
+      <c r="H22" s="5" t="inlineStr">
         <is>
           <t>20%</t>
         </is>
@@ -15546,7 +15546,7 @@
       </c>
       <c r="G31" s="5" t="inlineStr">
         <is>
-          <t>5522799</t>
+          <t>6633968</t>
         </is>
       </c>
       <c r="H31" s="5" t="inlineStr">
@@ -16439,40 +16439,40 @@
       </c>
     </row>
     <row r="54">
-      <c r="A54" s="7" t="inlineStr">
-        <is>
-          <t>01/03/2026</t>
-        </is>
-      </c>
-      <c r="B54" s="7" t="inlineStr">
+      <c r="A54" s="5" t="inlineStr">
+        <is>
+          <t>01/03/2026</t>
+        </is>
+      </c>
+      <c r="B54" s="5" t="inlineStr">
         <is>
           <t>René Furterer</t>
         </is>
       </c>
-      <c r="C54" s="7" t="inlineStr">
+      <c r="C54" s="5" t="inlineStr">
         <is>
           <t>Sublime Curl nutri-Activating Cream
 Creme Cabelo Leave-In Redefinidor de Caracóis
 100 ml</t>
         </is>
       </c>
-      <c r="D54" s="7" t="inlineStr">
+      <c r="D54" s="5" t="inlineStr">
         <is>
           <t>https://wells.pt/sublime-curl-nutri-activating-cream-5972165.html</t>
         </is>
       </c>
-      <c r="E54" s="7" t="inlineStr"/>
-      <c r="F54" s="8" t="inlineStr">
-        <is>
-          <t>Out of Stock</t>
-        </is>
-      </c>
-      <c r="G54" s="7" t="inlineStr">
+      <c r="E54" s="5" t="inlineStr"/>
+      <c r="F54" s="6" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
+      <c r="G54" s="5" t="inlineStr">
         <is>
           <t>5972165</t>
         </is>
       </c>
-      <c r="H54" s="7" t="inlineStr">
+      <c r="H54" s="5" t="inlineStr">
         <is>
           <t>28%</t>
         </is>
@@ -17253,40 +17253,40 @@
       </c>
     </row>
     <row r="74">
-      <c r="A74" s="7" t="inlineStr">
-        <is>
-          <t>01/03/2026</t>
-        </is>
-      </c>
-      <c r="B74" s="7" t="inlineStr">
+      <c r="A74" s="5" t="inlineStr">
+        <is>
+          <t>01/03/2026</t>
+        </is>
+      </c>
+      <c r="B74" s="5" t="inlineStr">
         <is>
           <t>René Furterer</t>
         </is>
       </c>
-      <c r="C74" s="7" t="inlineStr">
+      <c r="C74" s="5" t="inlineStr">
         <is>
           <t>Triphasic Texturizing Detangling Conditioner
 Condicionador Queda de Cabelo Texturarizante
 150 ml</t>
         </is>
       </c>
-      <c r="D74" s="7" t="inlineStr">
+      <c r="D74" s="5" t="inlineStr">
         <is>
           <t>https://wells.pt/triphasic-texturizing-detangling-conditioner-6856570.html</t>
         </is>
       </c>
-      <c r="E74" s="7" t="inlineStr"/>
-      <c r="F74" s="8" t="inlineStr">
-        <is>
-          <t>Out of Stock</t>
-        </is>
-      </c>
-      <c r="G74" s="7" t="inlineStr">
+      <c r="E74" s="5" t="inlineStr"/>
+      <c r="F74" s="6" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
+      <c r="G74" s="5" t="inlineStr">
         <is>
           <t>6856570</t>
         </is>
       </c>
-      <c r="H74" s="7" t="inlineStr">
+      <c r="H74" s="5" t="inlineStr">
         <is>
           <t>23%</t>
         </is>
@@ -17373,40 +17373,40 @@
       </c>
     </row>
     <row r="77">
-      <c r="A77" s="7" t="inlineStr">
-        <is>
-          <t>01/03/2026</t>
-        </is>
-      </c>
-      <c r="B77" s="7" t="inlineStr">
+      <c r="A77" s="3" t="inlineStr">
+        <is>
+          <t>01/03/2026</t>
+        </is>
+      </c>
+      <c r="B77" s="3" t="inlineStr">
         <is>
           <t>René Furterer</t>
         </is>
       </c>
-      <c r="C77" s="7" t="inlineStr">
+      <c r="C77" s="3" t="inlineStr">
         <is>
           <t>Volumea Volumizing Foam
 Espuma Volumizadora Cabelo Fino sem Volume
 200 ml</t>
         </is>
       </c>
-      <c r="D77" s="7" t="inlineStr">
+      <c r="D77" s="3" t="inlineStr">
         <is>
           <t>https://wells.pt/volumea-volumizing-foam-5520281.html</t>
         </is>
       </c>
-      <c r="E77" s="7" t="inlineStr"/>
-      <c r="F77" s="8" t="inlineStr">
-        <is>
-          <t>Out of Stock</t>
-        </is>
-      </c>
-      <c r="G77" s="7" t="inlineStr">
+      <c r="E77" s="3" t="inlineStr"/>
+      <c r="F77" s="4" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
+      <c r="G77" s="3" t="inlineStr">
         <is>
           <t>5520281</t>
         </is>
       </c>
-      <c r="H77" s="7" t="inlineStr">
+      <c r="H77" s="3" t="inlineStr">
         <is>
           <t>20%</t>
         </is>
@@ -20708,7 +20708,7 @@
       </c>
       <c r="E18" s="5" t="inlineStr">
         <is>
-          <t>3000998</t>
+          <t>3000993</t>
         </is>
       </c>
       <c r="F18" s="5" t="inlineStr">
@@ -21865,38 +21865,38 @@
       </c>
     </row>
     <row r="49">
-      <c r="A49" s="7" t="inlineStr">
+      <c r="A49" s="5" t="inlineStr">
         <is>
           <t>Klorane</t>
         </is>
       </c>
-      <c r="B49" s="7" t="inlineStr">
+      <c r="B49" s="5" t="inlineStr">
         <is>
           <t>Nettle Oil Control Shampoo
 Champô Ortiga BIO Purifica Cabelo Oleoso</t>
         </is>
       </c>
-      <c r="C49" s="7" t="inlineStr">
+      <c r="C49" s="5" t="inlineStr">
         <is>
           <t>400 ml</t>
         </is>
       </c>
-      <c r="D49" s="8" t="inlineStr">
-        <is>
-          <t>Out of Stock</t>
-        </is>
-      </c>
-      <c r="E49" s="7" t="inlineStr">
+      <c r="D49" s="6" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
+      <c r="E49" s="5" t="inlineStr">
         <is>
           <t>3688262</t>
         </is>
       </c>
-      <c r="F49" s="7" t="inlineStr">
+      <c r="F49" s="5" t="inlineStr">
         <is>
           <t>35%</t>
         </is>
       </c>
-      <c r="G49" s="7" t="inlineStr">
+      <c r="G49" s="5" t="inlineStr">
         <is>
           <t>https://wells.pt/nettle-oil-control-shampoo-343980.html</t>
         </is>
@@ -21941,38 +21941,38 @@
       </c>
     </row>
     <row r="51">
-      <c r="A51" s="7" t="inlineStr">
+      <c r="A51" s="3" t="inlineStr">
         <is>
           <t>Klorane</t>
         </is>
       </c>
-      <c r="B51" s="7" t="inlineStr">
+      <c r="B51" s="3" t="inlineStr">
         <is>
           <t>Oat &amp; Ceramide Ultra-Gentle Dry Shampoo
 Champô Seco Aveia Spray Suave Cabelo Normal</t>
         </is>
       </c>
-      <c r="C51" s="7" t="inlineStr">
+      <c r="C51" s="3" t="inlineStr">
         <is>
           <t>50 ml</t>
         </is>
       </c>
-      <c r="D51" s="8" t="inlineStr">
-        <is>
-          <t>Out of Stock</t>
-        </is>
-      </c>
-      <c r="E51" s="7" t="inlineStr">
+      <c r="D51" s="4" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
+      <c r="E51" s="3" t="inlineStr">
         <is>
           <t>7831152</t>
         </is>
       </c>
-      <c r="F51" s="7" t="inlineStr">
-        <is>
-          <t>25%</t>
-        </is>
-      </c>
-      <c r="G51" s="7" t="inlineStr">
+      <c r="F51" s="3" t="inlineStr">
+        <is>
+          <t>25%</t>
+        </is>
+      </c>
+      <c r="G51" s="3" t="inlineStr">
         <is>
           <t>https://wells.pt/oat-and-ceramide-ultra-gentle-dry-shampoo-341981.html</t>
         </is>
@@ -22420,7 +22420,7 @@
       </c>
       <c r="E63" s="3" t="inlineStr">
         <is>
-          <t>5522799</t>
+          <t>6633968</t>
         </is>
       </c>
       <c r="F63" s="3" t="inlineStr">

</xml_diff>